<commit_message>
Correção da falta de salvamento
</commit_message>
<xml_diff>
--- a/DadosMedicao.xlsx
+++ b/DadosMedicao.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Arquivos_de_Backup\Me\Universidade-UFSC\Curso_de_Engenharia_de_Controle_e_Automação\Sexta-fase\Metrologia\experimento2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Arquivos_de_Backup\Me\Universidade-UFSC\Curso_de_Engenharia_de_Controle_e_Automação\Sexta-fase\Metrologia\github-repository\Statistics-and-Probability\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FEFAC83-AA7E-43C5-BF78-AA423A04ABE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C42D25FA-5C19-4266-872A-0DA301494918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="13170" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>Numero medidas</t>
   </si>
@@ -111,9 +111,6 @@
     <t>Variação dos mensurandos</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>In</t>
   </si>
   <si>
@@ -145,13 +142,44 @@
   </si>
   <si>
     <t>Incerteza Padrão</t>
+  </si>
+  <si>
+    <t>Desvio Padrão Amostral</t>
+  </si>
+  <si>
+    <t>inf</t>
+  </si>
+  <si>
+    <t>Intervalo de Confiança</t>
+  </si>
+  <si>
+    <t>Graus de Liberdade Combinados</t>
+  </si>
+  <si>
+    <t>Incerteza padrão Combinada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t de student </t>
+  </si>
+  <si>
+    <t>Valor Base</t>
+  </si>
+  <si>
+    <t>Incerteza Expandida</t>
+  </si>
+  <si>
+    <t>Correção Combinada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="165" formatCode="#,##0.000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,8 +217,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="0.79998168889431442"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +334,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -495,7 +569,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -567,9 +641,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -581,16 +653,39 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -871,13 +966,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:R66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" customWidth="1"/>
+    <col min="7" max="7" width="32.7109375" customWidth="1"/>
     <col min="8" max="8" width="26.42578125" customWidth="1"/>
     <col min="9" max="9" width="23.28515625" customWidth="1"/>
     <col min="10" max="10" width="22.42578125" customWidth="1"/>
@@ -1392,345 +1488,762 @@
       <c r="E24">
         <v>1</v>
       </c>
-      <c r="M24" s="25"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="H25" s="24" t="s">
+      <c r="G25" s="23"/>
+      <c r="H25" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="I25" s="23"/>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="25"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="42"/>
+      <c r="K25" s="42"/>
+      <c r="L25" s="42"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="31"/>
-      <c r="B26" s="31" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
+      <c r="A26" s="29"/>
+      <c r="B26" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="G26" s="24" t="s">
+        <v>34</v>
+      </c>
       <c r="H26" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="I26" s="23"/>
+      <c r="I26" s="24"/>
       <c r="J26" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="K26" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="K26" s="24" t="s">
+      <c r="L26" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="L26" s="24" t="s">
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="32">
+        <v>250</v>
+      </c>
+      <c r="C27" s="32">
+        <v>365</v>
+      </c>
+      <c r="D27" s="32">
+        <v>2050</v>
+      </c>
+      <c r="G27" s="44">
+        <v>4</v>
+      </c>
+      <c r="H27" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="M26" s="25"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" s="35">
-        <v>250</v>
-      </c>
-      <c r="C27" s="35">
-        <v>365</v>
-      </c>
-      <c r="D27" s="35">
-        <v>2050</v>
-      </c>
-      <c r="H27" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="I27" s="29" t="s">
+      <c r="I27" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="J27" s="29">
-        <f>B37</f>
-        <v>-48.5</v>
-      </c>
-      <c r="K27" s="29">
-        <f t="shared" ref="K27:L27" si="0">C37</f>
+      <c r="J27" s="27">
+        <f>D36</f>
+        <v>-397</v>
+      </c>
+      <c r="K27" s="27">
+        <f>C36</f>
         <v>-71.600000000000023</v>
       </c>
-      <c r="L27" s="29">
-        <f t="shared" si="0"/>
-        <v>-397</v>
-      </c>
-      <c r="M27" s="26"/>
+      <c r="L27" s="27">
+        <f>B36</f>
+        <v>-48.600000000000023</v>
+      </c>
+      <c r="M27" s="25"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
-      <c r="B28" s="34">
+      <c r="A28" s="30">
+        <v>1</v>
+      </c>
+      <c r="B28" s="31">
         <v>299</v>
       </c>
-      <c r="C28" s="34">
+      <c r="C28" s="31">
         <v>436</v>
       </c>
-      <c r="D28" s="34">
+      <c r="D28" s="31">
         <v>2448</v>
       </c>
-      <c r="E28" s="33"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="29" t="s">
+      <c r="G28" s="44"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="J28" s="29">
-        <f>B35</f>
-        <v>0.54772255750516607</v>
-      </c>
-      <c r="K28" s="29">
-        <f t="shared" ref="K28:L28" si="1">C35</f>
+      <c r="J28" s="27">
+        <f>D34</f>
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="K28" s="27">
+        <f>C34</f>
         <v>0.54772255750516619</v>
       </c>
-      <c r="L28" s="29">
-        <f t="shared" si="1"/>
-        <v>0.70710678118654757</v>
-      </c>
-      <c r="M28" s="26"/>
+      <c r="L28" s="27">
+        <f>B34</f>
+        <v>0.54772255750516619</v>
+      </c>
+      <c r="M28" s="25"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
-      <c r="B29" s="34">
+      <c r="A29" s="30">
+        <f>A28+1</f>
+        <v>2</v>
+      </c>
+      <c r="B29" s="31">
         <v>299</v>
       </c>
-      <c r="C29" s="34">
+      <c r="C29" s="31">
         <v>437</v>
       </c>
-      <c r="D29" s="34">
+      <c r="D29" s="31">
         <v>2447</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="H29" s="30" t="s">
+      <c r="G29" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="H29" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="I29" s="29" t="s">
+      <c r="I29" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="J29" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="K29" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="L29" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="M29" s="26"/>
+      <c r="J29" s="26">
+        <v>0</v>
+      </c>
+      <c r="K29" s="26">
+        <v>0</v>
+      </c>
+      <c r="L29" s="26">
+        <v>0</v>
+      </c>
+      <c r="M29" s="25"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
-      <c r="B30" s="34">
+      <c r="A30" s="30">
+        <f t="shared" ref="A30:A32" si="0">A29+1</f>
+        <v>3</v>
+      </c>
+      <c r="B30" s="31">
         <v>298</v>
       </c>
-      <c r="C30" s="34">
+      <c r="C30" s="31">
         <v>437</v>
       </c>
-      <c r="D30" s="34">
+      <c r="D30" s="31">
         <v>2446</v>
       </c>
-      <c r="E30" s="33"/>
-      <c r="H30" s="30"/>
-      <c r="I30" s="29" t="s">
+      <c r="G30" s="44"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="J30" s="27">
-        <f>C44</f>
+      <c r="J30" s="26">
+        <f>C43</f>
         <v>0.28867513459481292</v>
       </c>
-      <c r="K30" s="27">
+      <c r="K30" s="26">
         <f>J30</f>
         <v>0.28867513459481292</v>
       </c>
-      <c r="L30" s="27">
+      <c r="L30" s="26">
         <f>K30</f>
         <v>0.28867513459481292</v>
       </c>
-      <c r="M30" s="26"/>
+      <c r="M30" s="25"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
-      <c r="B31" s="34">
+      <c r="A31" s="30">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="B31" s="31">
         <v>298</v>
       </c>
-      <c r="C31" s="34">
+      <c r="C31" s="31">
         <v>437</v>
       </c>
-      <c r="D31" s="34">
+      <c r="D31" s="31">
         <v>2447</v>
       </c>
-      <c r="E31" s="33"/>
-      <c r="H31" s="30" t="s">
+      <c r="G31" s="44">
+        <v>14</v>
+      </c>
+      <c r="H31" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="I31" s="29" t="s">
+      <c r="I31" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="J31" s="28" t="s">
+      <c r="J31" s="26">
+        <v>0</v>
+      </c>
+      <c r="K31" s="26">
+        <v>0</v>
+      </c>
+      <c r="L31" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" s="30">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="B32" s="31">
+        <v>299</v>
+      </c>
+      <c r="C32" s="31">
+        <v>436</v>
+      </c>
+      <c r="D32" s="31">
+        <v>2447</v>
+      </c>
+      <c r="G32" s="44"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="J32" s="26">
+        <f>D64</f>
+        <v>1.1126972805283735</v>
+      </c>
+      <c r="K32" s="26">
+        <f t="shared" ref="K32" si="1">C64</f>
+        <v>0.50709255283711008</v>
+      </c>
+      <c r="L32" s="26">
+        <f>B64</f>
+        <v>0.41403933560541262</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="32">
+        <f>AVERAGE(B28:B32)</f>
+        <v>298.60000000000002</v>
+      </c>
+      <c r="C33" s="32">
+        <f>AVERAGE(C28:C32)</f>
+        <v>436.6</v>
+      </c>
+      <c r="D33" s="32">
+        <f>AVERAGE(D28:D32)</f>
+        <v>2447</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="33">
+        <f>_xlfn.STDEV.S(B28:B32)</f>
+        <v>0.54772255750516619</v>
+      </c>
+      <c r="C34" s="33">
+        <f>_xlfn.STDEV.S(C28:C32)</f>
+        <v>0.54772255750516619</v>
+      </c>
+      <c r="D34" s="33">
+        <f>_xlfn.STDEV.S(D28:D32)</f>
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="H34" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="I34" s="47"/>
+      <c r="J34" s="47"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="32">
+        <f>B33-B27</f>
+        <v>48.600000000000023</v>
+      </c>
+      <c r="C35" s="32">
+        <f>C33-C27</f>
+        <v>71.600000000000023</v>
+      </c>
+      <c r="D35" s="32">
+        <f>D33-D27</f>
+        <v>397</v>
+      </c>
+      <c r="G35" s="45"/>
+      <c r="H35" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="K31" s="28" t="s">
+      <c r="I35" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="J35" s="48" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="34">
+        <f>-B35</f>
+        <v>-48.600000000000023</v>
+      </c>
+      <c r="C36" s="34">
+        <f t="shared" ref="C36:D36" si="2">-C35</f>
+        <v>-71.600000000000023</v>
+      </c>
+      <c r="D36" s="34">
+        <f t="shared" si="2"/>
+        <v>-397</v>
+      </c>
+      <c r="G36" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="H36" s="43">
+        <f>(H37^4)/((J28^4/$G$27) + (J32^4/$G$31))</f>
+        <v>19.289346674514416</v>
+      </c>
+      <c r="I36" s="43">
+        <f>(I37^4)/((K28^4/$G$27) + (K32^4/$G$31))</f>
+        <v>15.068481332738367</v>
+      </c>
+      <c r="J36" s="43">
+        <f>(J37^4)/((L28^4/$G$27) + (L32^4/$G$31))</f>
+        <v>12.511045267489708</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="34">
+        <v>5</v>
+      </c>
+      <c r="C37" s="34">
+        <v>4</v>
+      </c>
+      <c r="D37" s="34">
+        <v>4</v>
+      </c>
+      <c r="G37" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="H37" s="43">
+        <f>SQRT(J28^2 + J30^2 + J32^2)</f>
+        <v>1.3496031162636559</v>
+      </c>
+      <c r="I37" s="43">
+        <f>SQRT(K28^2 + K30^2 + K32^2)</f>
+        <v>0.80029756370751925</v>
+      </c>
+      <c r="J37" s="43">
+        <f>SQRT(L28^2 + L30^2 + L32^2)</f>
+        <v>0.74482340508465827</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="29"/>
+      <c r="B38" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="D38" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="L31" s="28" t="s">
+      <c r="G38" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="H38" s="43">
+        <f>J27+J29+J31</f>
+        <v>-397</v>
+      </c>
+      <c r="I38" s="43">
+        <f>K27+K29+K31</f>
+        <v>-71.600000000000023</v>
+      </c>
+      <c r="J38" s="43">
+        <f>L27+L29+L31</f>
+        <v>-48.600000000000023</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="G39" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="H39" s="49">
+        <v>2.133</v>
+      </c>
+      <c r="I39" s="49">
+        <v>2.169</v>
+      </c>
+      <c r="J39" s="49">
+        <v>2.2120000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="35"/>
+      <c r="G40" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="H40" s="43">
+        <f>D63+H38</f>
+        <v>1654.6666666666665</v>
+      </c>
+      <c r="I40" s="50">
+        <f>C63+I38</f>
+        <v>293.79999999999995</v>
+      </c>
+      <c r="J40" s="50">
+        <f>B63+J38</f>
+        <v>198.2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="36" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="37">
+        <v>1</v>
+      </c>
+      <c r="G41" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="H41" s="43">
+        <f>H37*H39</f>
+        <v>2.8787034469903783</v>
+      </c>
+      <c r="I41" s="43">
+        <f>I37*I39</f>
+        <v>1.7358454156816092</v>
+      </c>
+      <c r="J41" s="43">
+        <f>J37*J39</f>
+        <v>1.6475493720472643</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="37">
+        <f>C41/2</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B43" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C43" s="37">
+        <f>C42/SQRT(3)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J44" s="51"/>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="39"/>
+      <c r="B47" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" s="39" t="s">
+        <v>29</v>
+      </c>
+      <c r="D47" s="39" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
-      <c r="B32" s="34">
-        <v>299</v>
-      </c>
-      <c r="C32" s="34">
-        <v>436</v>
-      </c>
-      <c r="D32" s="34">
-        <v>2447</v>
-      </c>
-      <c r="E32" s="33"/>
-      <c r="H32" s="30"/>
-      <c r="I32" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="27"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
-      <c r="B33" s="34">
-        <v>298</v>
-      </c>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="32" t="s">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="39">
+        <v>1</v>
+      </c>
+      <c r="B48" s="40">
+        <v>247</v>
+      </c>
+      <c r="C48" s="40">
+        <v>365</v>
+      </c>
+      <c r="D48" s="40">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="39">
+        <f>A48+1</f>
+        <v>2</v>
+      </c>
+      <c r="B49" s="40">
+        <v>247</v>
+      </c>
+      <c r="C49" s="40">
+        <v>365</v>
+      </c>
+      <c r="D49" s="40">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="39">
+        <f t="shared" ref="A50:A62" si="3">A49+1</f>
+        <v>3</v>
+      </c>
+      <c r="B50" s="40">
+        <v>247</v>
+      </c>
+      <c r="C50" s="40">
+        <v>366</v>
+      </c>
+      <c r="D50" s="40">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="39">
+        <f t="shared" si="3"/>
+        <v>4</v>
+      </c>
+      <c r="B51" s="40">
+        <v>247</v>
+      </c>
+      <c r="C51" s="40">
+        <v>366</v>
+      </c>
+      <c r="D51" s="40">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="39">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="B52" s="40">
+        <v>246</v>
+      </c>
+      <c r="C52" s="40">
+        <v>365</v>
+      </c>
+      <c r="D52" s="40">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="39">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+      <c r="B53" s="40">
+        <v>246</v>
+      </c>
+      <c r="C53" s="40">
+        <v>365</v>
+      </c>
+      <c r="D53" s="40">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="39">
+        <f t="shared" si="3"/>
+        <v>7</v>
+      </c>
+      <c r="B54" s="40">
+        <v>246</v>
+      </c>
+      <c r="C54" s="40">
+        <v>365</v>
+      </c>
+      <c r="D54" s="40">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="39">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="B55" s="40">
+        <v>247</v>
+      </c>
+      <c r="C55" s="40">
+        <v>366</v>
+      </c>
+      <c r="D55" s="40">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="39">
+        <f t="shared" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="B56" s="40">
+        <v>247</v>
+      </c>
+      <c r="C56" s="40">
+        <v>365</v>
+      </c>
+      <c r="D56" s="40">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="39">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="B57" s="40">
+        <v>247</v>
+      </c>
+      <c r="C57" s="40">
+        <v>366</v>
+      </c>
+      <c r="D57" s="40">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="39">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="B58" s="40">
+        <v>247</v>
+      </c>
+      <c r="C58" s="40">
+        <v>366</v>
+      </c>
+      <c r="D58" s="40">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="39">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="B59" s="40">
+        <v>247</v>
+      </c>
+      <c r="C59" s="40">
+        <v>366</v>
+      </c>
+      <c r="D59" s="40">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="39">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="B60" s="40">
+        <v>247</v>
+      </c>
+      <c r="C60" s="40">
+        <v>365</v>
+      </c>
+      <c r="D60" s="40">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="39">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="B61" s="40">
+        <v>247</v>
+      </c>
+      <c r="C61" s="40">
+        <v>365</v>
+      </c>
+      <c r="D61" s="40">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="39">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="B62" s="40">
+        <v>247</v>
+      </c>
+      <c r="C62" s="40">
+        <v>365</v>
+      </c>
+      <c r="D62" s="40">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="35">
-        <f>AVERAGE(B28:B33)</f>
-        <v>298.5</v>
-      </c>
-      <c r="C34" s="35">
-        <f t="shared" ref="C34:D34" si="2">AVERAGE(C28:C33)</f>
-        <v>436.6</v>
-      </c>
-      <c r="D34" s="35">
-        <f t="shared" si="2"/>
-        <v>2447</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="B35" s="36">
-        <f>_xlfn.STDEV.S(B28:B33)</f>
-        <v>0.54772255750516607</v>
-      </c>
-      <c r="C35" s="36">
-        <f t="shared" ref="C35:D35" si="3">_xlfn.STDEV.S(C28:C33)</f>
-        <v>0.54772255750516619</v>
-      </c>
-      <c r="D35" s="36">
-        <f t="shared" si="3"/>
-        <v>0.70710678118654757</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B36" s="35">
-        <f>B34-B27</f>
-        <v>48.5</v>
-      </c>
-      <c r="C36" s="35">
-        <f t="shared" ref="C36:D36" si="4">C34-C27</f>
-        <v>71.600000000000023</v>
-      </c>
-      <c r="D36" s="35">
+      <c r="B63" s="39">
+        <f>AVERAGE(B48:B62)</f>
+        <v>246.8</v>
+      </c>
+      <c r="C63" s="39">
+        <f t="shared" ref="C63:D63" si="4">AVERAGE(C48:C62)</f>
+        <v>365.4</v>
+      </c>
+      <c r="D63" s="39">
         <f t="shared" si="4"/>
-        <v>397</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="37">
-        <f>-B36</f>
-        <v>-48.5</v>
-      </c>
-      <c r="C37" s="37">
-        <f t="shared" ref="C37:D37" si="5">-C36</f>
-        <v>-71.600000000000023</v>
-      </c>
-      <c r="D37" s="37">
+        <v>2051.6666666666665</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B64" s="39">
+        <f>STDEVA(B48:B62)</f>
+        <v>0.41403933560541262</v>
+      </c>
+      <c r="C64" s="39">
+        <f t="shared" ref="C64:D64" si="5">STDEVA(C48:C62)</f>
+        <v>0.50709255283711008</v>
+      </c>
+      <c r="D64" s="39">
         <f t="shared" si="5"/>
-        <v>-397</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" s="37">
-        <v>5</v>
-      </c>
-      <c r="C38" s="37">
-        <v>4</v>
-      </c>
-      <c r="D38" s="37">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="31"/>
-      <c r="B39" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="C39" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="D39" s="31" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="C41" s="38"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="39" t="s">
-        <v>37</v>
-      </c>
-      <c r="C42" s="40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B43" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="C43" s="40">
-        <f>C42/2</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="C44" s="40">
-        <f>C43/SQRT(3)</f>
-        <v>0.28867513459481292</v>
-      </c>
+        <v>1.1126972805283735</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="41"/>
+      <c r="B65" s="41"/>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="41"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="H25:L25"/>
+    <mergeCell ref="H34:J34"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>